<commit_message>
Sanitize public code package for peer review
</commit_message>
<xml_diff>
--- a/supporting_information/S1_Table.xlsx
+++ b/supporting_information/S1_Table.xlsx
@@ -20114,7 +20114,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\results\tables\deep_axis_tcga_immune_associations.tsv</t>
+          <t>project-root:\spatial_escc_workflow\results\tables\deep_axis_tcga_immune_associations.tsv</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -20159,7 +20159,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\geo\GSE47404\GSE47404_series_matrix.txt.gz</t>
+          <t>project-root:\spatial_escc_workflow\data\geo\GSE47404\GSE47404_series_matrix.txt.gz</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -20204,7 +20204,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\geo\GSE53625\GSE53625_series_matrix.txt.gz</t>
+          <t>project-root:\spatial_escc_workflow\data\geo\GSE53625\GSE53625_series_matrix.txt.gz</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -20249,7 +20249,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\geo\GSE53625\GSM1296956_first_raw_member.txt.gz</t>
+          <t>project-root:\spatial_escc_workflow\data\geo\GSE53625\GSM1296956_first_raw_member.txt.gz</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -20294,7 +20294,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\results\tables\gse53625_ensembl_sequence_index.tsv</t>
+          <t>project-root:\spatial_escc_workflow\results\tables\gse53625_ensembl_sequence_index.tsv</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -20339,7 +20339,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\open_source_tables\HRA003627_NatCommun2023_source_data.xlsx</t>
+          <t>project-root:\spatial_escc_workflow\data\open_source_tables\HRA003627_NatCommun2023_source_data.xlsx</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -20384,7 +20384,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\open_source_tables\HRA008846_TableS3_DEG.xlsx</t>
+          <t>project-root:\spatial_escc_workflow\data\open_source_tables\HRA008846_TableS3_DEG.xlsx</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -20429,7 +20429,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\open_source_tables\HRA008846_TableS4_cell_abundance.xlsx</t>
+          <t>project-root:\spatial_escc_workflow\data\open_source_tables\HRA008846_TableS4_cell_abundance.xlsx</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -20474,7 +20474,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\open_source_tables\HRA008846_TableS6_ligand_receptor.xlsx</t>
+          <t>project-root:\spatial_escc_workflow\data\open_source_tables\HRA008846_TableS6_ligand_receptor.xlsx</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -20519,7 +20519,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\gdsc\GDSC2_fitted_dose_response_27Oct23.xlsx</t>
+          <t>project-root:\spatial_escc_workflow\data\gdsc\GDSC2_fitted_dose_response_27Oct23.xlsx</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -20656,7 +20656,6 @@
       <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>CD8A,CD8B,GZMB,PRF1,NKG7,GNLY</t>
@@ -20703,7 +20702,6 @@
       <c r="G3" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>FOXP3,IL2RA,CTLA4,IKZF2,CCR8</t>
@@ -20750,7 +20748,6 @@
       <c r="G4" t="n">
         <v>0</v>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>PDCD1,CD274,CTLA4,LAG3,HAVCR2,TIGIT</t>
@@ -20797,7 +20794,6 @@
       <c r="G5" t="n">
         <v>0</v>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
@@ -20844,7 +20840,6 @@
       <c r="G6" t="n">
         <v>0</v>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>CD68,CD163,MRC1,CSF1R,MSR1</t>
@@ -20891,7 +20886,6 @@
       <c r="G7" t="n">
         <v>0</v>
       </c>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>FAP,ACTA2,COL1A1,COL1A2,PDGFRB,POSTN</t>
@@ -20938,7 +20932,6 @@
       <c r="G8" t="n">
         <v>0</v>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>PECAM1,VWF,KDR,CDH5,ENG</t>
@@ -20985,7 +20978,6 @@
       <c r="G9" t="n">
         <v>0</v>
       </c>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>S100A8,S100A9,FCGR3B,CXCR2,CSF3R</t>
@@ -21032,7 +21024,6 @@
       <c r="G10" t="n">
         <v>0</v>
       </c>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>IFNG,CXCL9,CXCL10,STAT1,IRF1,IDO1,CD274</t>
@@ -21181,7 +21172,6 @@
       <c r="G13" t="n">
         <v>0</v>
       </c>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>VIM,SNAI1,SNAI2,ZEB1,ZEB2,CDH2,FN1,ITGA5,MMP2</t>
@@ -21228,7 +21218,6 @@
       <c r="G14" t="n">
         <v>0</v>
       </c>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>COL1A1,COL1A2,COL3A1,FN1,POSTN,LOX,MMP2,MMP9</t>
@@ -21275,7 +21264,6 @@
       <c r="G15" t="n">
         <v>0</v>
       </c>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>HIF1A,VEGFA,CA9,SLC2A1,LDHA,PDK1</t>
@@ -21322,7 +21310,6 @@
       <c r="G16" t="n">
         <v>0</v>
       </c>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>MKI67,PCNA,TOP2A,CCNB1,MCM2,MCM6</t>
@@ -21369,7 +21356,6 @@
       <c r="G17" t="n">
         <v>0</v>
       </c>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>BAX,CASP3,CASP8,FAS,BCL2L11,PMAIP1</t>
@@ -21416,7 +21402,6 @@
       <c r="G18" t="n">
         <v>0</v>
       </c>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
@@ -21463,7 +21448,6 @@
       <c r="G19" t="n">
         <v>0</v>
       </c>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>CD274,PDCD1,CTLA4,LAG3,TIGIT,HAVCR2</t>
@@ -21510,7 +21494,6 @@
       <c r="G20" t="n">
         <v>0</v>
       </c>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>CD8A,CD8B,GZMB,PRF1,NKG7,GNLY</t>
@@ -21557,7 +21540,6 @@
       <c r="G21" t="n">
         <v>0</v>
       </c>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>FOXP3,IL2RA,CTLA4,IKZF2,CCR8</t>
@@ -21604,7 +21586,6 @@
       <c r="G22" t="n">
         <v>0</v>
       </c>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>PDCD1,CD274,CTLA4,LAG3,HAVCR2,TIGIT</t>
@@ -21651,7 +21632,6 @@
       <c r="G23" t="n">
         <v>0</v>
       </c>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
@@ -21698,7 +21678,6 @@
       <c r="G24" t="n">
         <v>0</v>
       </c>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>CD68,CD163,MRC1,CSF1R,MSR1</t>
@@ -21796,7 +21775,6 @@
       <c r="G26" t="n">
         <v>0</v>
       </c>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>PECAM1,VWF,KDR,CDH5,ENG</t>
@@ -21843,7 +21821,6 @@
       <c r="G27" t="n">
         <v>0</v>
       </c>
-      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
           <t>S100A8,S100A9,FCGR3B,CXCR2,CSF3R</t>
@@ -21890,7 +21867,6 @@
       <c r="G28" t="n">
         <v>0</v>
       </c>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>IFNG,CXCL9,CXCL10,STAT1,IRF1,IDO1,CD274</t>
@@ -21937,7 +21913,6 @@
       <c r="G29" t="n">
         <v>0</v>
       </c>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>PIK3CA,PIK3CB,AKT1,AKT2,MTOR,RPS6KB1,EIF4EBP1</t>
@@ -22035,7 +22010,6 @@
       <c r="G31" t="n">
         <v>0</v>
       </c>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>VIM,SNAI1,SNAI2,ZEB1,ZEB2,CDH2,FN1,ITGA5,MMP2</t>
@@ -22133,7 +22107,6 @@
       <c r="G33" t="n">
         <v>0</v>
       </c>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>HIF1A,VEGFA,CA9,SLC2A1,LDHA,PDK1</t>
@@ -22180,7 +22153,6 @@
       <c r="G34" t="n">
         <v>0</v>
       </c>
-      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>MKI67,PCNA,TOP2A,CCNB1,MCM2,MCM6</t>
@@ -22227,7 +22199,6 @@
       <c r="G35" t="n">
         <v>0</v>
       </c>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>BAX,CASP3,CASP8,FAS,BCL2L11,PMAIP1</t>
@@ -22274,7 +22245,6 @@
       <c r="G36" t="n">
         <v>0</v>
       </c>
-      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
@@ -22321,7 +22291,6 @@
       <c r="G37" t="n">
         <v>0</v>
       </c>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>CD274,PDCD1,CTLA4,LAG3,TIGIT,HAVCR2</t>
@@ -22574,7 +22543,6 @@
           <t>CD8A,CD8B,GZMB,PRF1,NKG7,GNLY</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
         <v>0</v>
       </c>
@@ -22679,7 +22647,6 @@
           <t>FOXP3,IL2RA,CTLA4,IKZF2,CCR8</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
         <v>0</v>
       </c>
@@ -22784,7 +22751,6 @@
           <t>PDCD1,CD274,CTLA4,LAG3,HAVCR2,TIGIT</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
         <v>0</v>
       </c>
@@ -22889,7 +22855,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
       <c r="O5" t="n">
         <v>0</v>
       </c>
@@ -22994,7 +22959,6 @@
           <t>CD68,CD163,MRC1,CSF1R,MSR1</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
       <c r="O6" t="n">
         <v>0</v>
       </c>
@@ -23099,7 +23063,6 @@
           <t>FAP,ACTA2,COL1A1,COL1A2,PDGFRB,POSTN</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
       <c r="O7" t="n">
         <v>0</v>
       </c>
@@ -23204,7 +23167,6 @@
           <t>PECAM1,VWF,KDR,CDH5,ENG</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
       <c r="O8" t="n">
         <v>0</v>
       </c>
@@ -23309,7 +23271,6 @@
           <t>S100A8,S100A9,FCGR3B,CXCR2,CSF3R</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
       <c r="O9" t="n">
         <v>0</v>
       </c>
@@ -23414,7 +23375,6 @@
           <t>IFNG,CXCL9,CXCL10,STAT1,IRF1,IDO1,CD274</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
       <c r="O10" t="n">
         <v>0</v>
       </c>
@@ -23737,7 +23697,6 @@
           <t>VIM,SNAI1,SNAI2,ZEB1,ZEB2,CDH2,FN1,ITGA5,MMP2</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
       <c r="O13" t="n">
         <v>0</v>
       </c>
@@ -23842,7 +23801,6 @@
           <t>COL1A1,COL1A2,COL3A1,FN1,POSTN,LOX,MMP2,MMP9</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr"/>
       <c r="O14" t="n">
         <v>0</v>
       </c>
@@ -23947,7 +23905,6 @@
           <t>HIF1A,VEGFA,CA9,SLC2A1,LDHA,PDK1</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
       <c r="O15" t="n">
         <v>0</v>
       </c>
@@ -24052,7 +24009,6 @@
           <t>MKI67,PCNA,TOP2A,CCNB1,MCM2,MCM6</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr"/>
       <c r="O16" t="n">
         <v>0</v>
       </c>
@@ -24157,7 +24113,6 @@
           <t>BAX,CASP3,CASP8,FAS,BCL2L11,PMAIP1</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
       <c r="O17" t="n">
         <v>0</v>
       </c>
@@ -24262,7 +24217,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
       <c r="O18" t="n">
         <v>0</v>
       </c>
@@ -24367,7 +24321,6 @@
           <t>CD274,PDCD1,CTLA4,LAG3,TIGIT,HAVCR2</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
       <c r="O19" t="n">
         <v>0</v>
       </c>
@@ -24472,7 +24425,6 @@
           <t>CD8A,CD8B,GZMB,PRF1,NKG7,GNLY</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
       <c r="O20" t="n">
         <v>0</v>
       </c>
@@ -24577,7 +24529,6 @@
           <t>FOXP3,IL2RA,CTLA4,IKZF2,CCR8</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
       <c r="O21" t="n">
         <v>0</v>
       </c>
@@ -24682,7 +24633,6 @@
           <t>PDCD1,CD274,CTLA4,LAG3,HAVCR2,TIGIT</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr"/>
       <c r="O22" t="n">
         <v>0</v>
       </c>
@@ -24787,7 +24737,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
       <c r="O23" t="n">
         <v>0</v>
       </c>
@@ -24892,7 +24841,6 @@
           <t>CD68,CD163,MRC1,CSF1R,MSR1</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
       <c r="O24" t="n">
         <v>0</v>
       </c>
@@ -25106,7 +25054,6 @@
           <t>PECAM1,VWF,KDR,CDH5,ENG</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
       <c r="O26" t="n">
         <v>0</v>
       </c>
@@ -25211,7 +25158,6 @@
           <t>S100A8,S100A9,FCGR3B,CXCR2,CSF3R</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
       <c r="O27" t="n">
         <v>0</v>
       </c>
@@ -25316,7 +25262,6 @@
           <t>IFNG,CXCL9,CXCL10,STAT1,IRF1,IDO1,CD274</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr"/>
       <c r="O28" t="n">
         <v>0</v>
       </c>
@@ -25421,7 +25366,6 @@
           <t>PIK3CA,PIK3CB,AKT1,AKT2,MTOR,RPS6KB1,EIF4EBP1</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
       <c r="O29" t="n">
         <v>0</v>
       </c>
@@ -25635,7 +25579,6 @@
           <t>VIM,SNAI1,SNAI2,ZEB1,ZEB2,CDH2,FN1,ITGA5,MMP2</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
       <c r="O31" t="n">
         <v>0</v>
       </c>
@@ -25849,7 +25792,6 @@
           <t>HIF1A,VEGFA,CA9,SLC2A1,LDHA,PDK1</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
       <c r="O33" t="n">
         <v>0</v>
       </c>
@@ -25954,7 +25896,6 @@
           <t>MKI67,PCNA,TOP2A,CCNB1,MCM2,MCM6</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr"/>
       <c r="O34" t="n">
         <v>0</v>
       </c>
@@ -26059,7 +26000,6 @@
           <t>BAX,CASP3,CASP8,FAS,BCL2L11,PMAIP1</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
       <c r="O35" t="n">
         <v>0</v>
       </c>
@@ -26164,7 +26104,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr"/>
       <c r="O36" t="n">
         <v>0</v>
       </c>
@@ -26269,7 +26208,6 @@
           <t>CD274,PDCD1,CTLA4,LAG3,TIGIT,HAVCR2</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr"/>
       <c r="O37" t="n">
         <v>0</v>
       </c>
@@ -26374,7 +26312,6 @@
           <t>CD8A,CD8B,GZMB,PRF1,NKG7,GNLY</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr"/>
       <c r="O38" t="n">
         <v>0</v>
       </c>
@@ -26479,7 +26416,6 @@
           <t>FOXP3,IL2RA,CTLA4,IKZF2,CCR8</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr"/>
       <c r="O39" t="n">
         <v>0</v>
       </c>
@@ -26584,7 +26520,6 @@
           <t>PDCD1,CD274,CTLA4,LAG3,HAVCR2,TIGIT</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr"/>
       <c r="O40" t="n">
         <v>0</v>
       </c>
@@ -26689,7 +26624,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr"/>
       <c r="O41" t="n">
         <v>0</v>
       </c>
@@ -26794,7 +26728,6 @@
           <t>CD68,CD163,MRC1,CSF1R,MSR1</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr"/>
       <c r="O42" t="n">
         <v>0</v>
       </c>
@@ -26899,7 +26832,6 @@
           <t>FAP,ACTA2,COL1A1,COL1A2,PDGFRB,POSTN</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr"/>
       <c r="O43" t="n">
         <v>0</v>
       </c>
@@ -27004,7 +26936,6 @@
           <t>PECAM1,VWF,KDR,CDH5,ENG</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr"/>
       <c r="O44" t="n">
         <v>0</v>
       </c>
@@ -27109,7 +27040,6 @@
           <t>S100A8,S100A9,FCGR3B,CXCR2,CSF3R</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr"/>
       <c r="O45" t="n">
         <v>0</v>
       </c>
@@ -27214,7 +27144,6 @@
           <t>IFNG,CXCL9,CXCL10,STAT1,IRF1,IDO1,CD274</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr"/>
       <c r="O46" t="n">
         <v>0</v>
       </c>
@@ -27537,7 +27466,6 @@
           <t>VIM,SNAI1,SNAI2,ZEB1,ZEB2,CDH2,FN1,ITGA5,MMP2</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr"/>
       <c r="O49" t="n">
         <v>0</v>
       </c>
@@ -27642,7 +27570,6 @@
           <t>COL1A1,COL1A2,COL3A1,FN1,POSTN,LOX,MMP2,MMP9</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr"/>
       <c r="O50" t="n">
         <v>0</v>
       </c>
@@ -27747,7 +27674,6 @@
           <t>HIF1A,VEGFA,CA9,SLC2A1,LDHA,PDK1</t>
         </is>
       </c>
-      <c r="N51" t="inlineStr"/>
       <c r="O51" t="n">
         <v>0</v>
       </c>
@@ -27852,7 +27778,6 @@
           <t>MKI67,PCNA,TOP2A,CCNB1,MCM2,MCM6</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr"/>
       <c r="O52" t="n">
         <v>0</v>
       </c>
@@ -27957,7 +27882,6 @@
           <t>BAX,CASP3,CASP8,FAS,BCL2L11,PMAIP1</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr"/>
       <c r="O53" t="n">
         <v>0</v>
       </c>
@@ -28062,7 +27986,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr"/>
       <c r="O54" t="n">
         <v>0</v>
       </c>
@@ -28167,7 +28090,6 @@
           <t>CD274,PDCD1,CTLA4,LAG3,TIGIT,HAVCR2</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr"/>
       <c r="O55" t="n">
         <v>0</v>
       </c>
@@ -28272,7 +28194,6 @@
           <t>CD8A,CD8B,GZMB,PRF1,NKG7,GNLY</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr"/>
       <c r="O56" t="n">
         <v>0</v>
       </c>
@@ -28377,7 +28298,6 @@
           <t>FOXP3,IL2RA,CTLA4,IKZF2,CCR8</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr"/>
       <c r="O57" t="n">
         <v>0</v>
       </c>
@@ -28482,7 +28402,6 @@
           <t>PDCD1,CD274,CTLA4,LAG3,HAVCR2,TIGIT</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr"/>
       <c r="O58" t="n">
         <v>0</v>
       </c>
@@ -28587,7 +28506,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr"/>
       <c r="O59" t="n">
         <v>0</v>
       </c>
@@ -28692,7 +28610,6 @@
           <t>CD68,CD163,MRC1,CSF1R,MSR1</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr"/>
       <c r="O60" t="n">
         <v>0</v>
       </c>
@@ -28906,7 +28823,6 @@
           <t>PECAM1,VWF,KDR,CDH5,ENG</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr"/>
       <c r="O62" t="n">
         <v>0</v>
       </c>
@@ -29011,7 +28927,6 @@
           <t>S100A8,S100A9,FCGR3B,CXCR2,CSF3R</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr"/>
       <c r="O63" t="n">
         <v>0</v>
       </c>
@@ -29116,7 +29031,6 @@
           <t>IFNG,CXCL9,CXCL10,STAT1,IRF1,IDO1,CD274</t>
         </is>
       </c>
-      <c r="N64" t="inlineStr"/>
       <c r="O64" t="n">
         <v>0</v>
       </c>
@@ -29221,7 +29135,6 @@
           <t>PIK3CA,PIK3CB,AKT1,AKT2,MTOR,RPS6KB1,EIF4EBP1</t>
         </is>
       </c>
-      <c r="N65" t="inlineStr"/>
       <c r="O65" t="n">
         <v>0</v>
       </c>
@@ -29435,7 +29348,6 @@
           <t>VIM,SNAI1,SNAI2,ZEB1,ZEB2,CDH2,FN1,ITGA5,MMP2</t>
         </is>
       </c>
-      <c r="N67" t="inlineStr"/>
       <c r="O67" t="n">
         <v>0</v>
       </c>
@@ -29649,7 +29561,6 @@
           <t>HIF1A,VEGFA,CA9,SLC2A1,LDHA,PDK1</t>
         </is>
       </c>
-      <c r="N69" t="inlineStr"/>
       <c r="O69" t="n">
         <v>0</v>
       </c>
@@ -29754,7 +29665,6 @@
           <t>MKI67,PCNA,TOP2A,CCNB1,MCM2,MCM6</t>
         </is>
       </c>
-      <c r="N70" t="inlineStr"/>
       <c r="O70" t="n">
         <v>0</v>
       </c>
@@ -29859,7 +29769,6 @@
           <t>BAX,CASP3,CASP8,FAS,BCL2L11,PMAIP1</t>
         </is>
       </c>
-      <c r="N71" t="inlineStr"/>
       <c r="O71" t="n">
         <v>0</v>
       </c>
@@ -29964,7 +29873,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N72" t="inlineStr"/>
       <c r="O72" t="n">
         <v>0</v>
       </c>
@@ -30069,7 +29977,6 @@
           <t>CD274,PDCD1,CTLA4,LAG3,TIGIT,HAVCR2</t>
         </is>
       </c>
-      <c r="N73" t="inlineStr"/>
       <c r="O73" t="n">
         <v>0</v>
       </c>
@@ -30429,7 +30336,6 @@
           <t>CD8A,CD8B,GZMB,PRF1,NKG7,GNLY</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
         <v>0</v>
       </c>
@@ -30526,7 +30432,6 @@
           <t>FOXP3,IL2RA,CTLA4,IKZF2,CCR8</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
         <v>0</v>
       </c>
@@ -30623,7 +30528,6 @@
           <t>PDCD1,CD274,CTLA4,LAG3,HAVCR2,TIGIT</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
         <v>0</v>
       </c>
@@ -30720,7 +30624,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
       <c r="O5" t="n">
         <v>0</v>
       </c>
@@ -30817,7 +30720,6 @@
           <t>CD68,CD163,MRC1,CSF1R,MSR1</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr"/>
       <c r="O6" t="n">
         <v>0</v>
       </c>
@@ -30914,7 +30816,6 @@
           <t>FAP,ACTA2,COL1A1,COL1A2,PDGFRB,POSTN</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr"/>
       <c r="O7" t="n">
         <v>0</v>
       </c>
@@ -31011,7 +30912,6 @@
           <t>PECAM1,VWF,KDR,CDH5,ENG</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
       <c r="O8" t="n">
         <v>0</v>
       </c>
@@ -31108,7 +31008,6 @@
           <t>S100A8,S100A9,FCGR3B,CXCR2,CSF3R</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
       <c r="O9" t="n">
         <v>0</v>
       </c>
@@ -31205,7 +31104,6 @@
           <t>IFNG,CXCL9,CXCL10,STAT1,IRF1,IDO1,CD274</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr"/>
       <c r="O10" t="n">
         <v>0</v>
       </c>
@@ -31504,7 +31402,6 @@
           <t>VIM,SNAI1,SNAI2,ZEB1,ZEB2,CDH2,FN1,ITGA5,MMP2</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
       <c r="O13" t="n">
         <v>0</v>
       </c>
@@ -31601,7 +31498,6 @@
           <t>COL1A1,COL1A2,COL3A1,FN1,POSTN,LOX,MMP2,MMP9</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr"/>
       <c r="O14" t="n">
         <v>0</v>
       </c>
@@ -31698,7 +31594,6 @@
           <t>HIF1A,VEGFA,CA9,SLC2A1,LDHA,PDK1</t>
         </is>
       </c>
-      <c r="N15" t="inlineStr"/>
       <c r="O15" t="n">
         <v>0</v>
       </c>
@@ -31795,7 +31690,6 @@
           <t>MKI67,PCNA,TOP2A,CCNB1,MCM2,MCM6</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr"/>
       <c r="O16" t="n">
         <v>0</v>
       </c>
@@ -31892,7 +31786,6 @@
           <t>BAX,CASP3,CASP8,FAS,BCL2L11,PMAIP1</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
       <c r="O17" t="n">
         <v>0</v>
       </c>
@@ -31989,7 +31882,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N18" t="inlineStr"/>
       <c r="O18" t="n">
         <v>0</v>
       </c>
@@ -32086,7 +31978,6 @@
           <t>CD274,PDCD1,CTLA4,LAG3,TIGIT,HAVCR2</t>
         </is>
       </c>
-      <c r="N19" t="inlineStr"/>
       <c r="O19" t="n">
         <v>0</v>
       </c>
@@ -32183,7 +32074,6 @@
           <t>CD8A,CD8B,GZMB,PRF1,NKG7,GNLY</t>
         </is>
       </c>
-      <c r="N20" t="inlineStr"/>
       <c r="O20" t="n">
         <v>0</v>
       </c>
@@ -32280,7 +32170,6 @@
           <t>FOXP3,IL2RA,CTLA4,IKZF2,CCR8</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
       <c r="O21" t="n">
         <v>0</v>
       </c>
@@ -32377,7 +32266,6 @@
           <t>PDCD1,CD274,CTLA4,LAG3,HAVCR2,TIGIT</t>
         </is>
       </c>
-      <c r="N22" t="inlineStr"/>
       <c r="O22" t="n">
         <v>0</v>
       </c>
@@ -32474,7 +32362,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N23" t="inlineStr"/>
       <c r="O23" t="n">
         <v>0</v>
       </c>
@@ -32571,7 +32458,6 @@
           <t>CD68,CD163,MRC1,CSF1R,MSR1</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
       <c r="O24" t="n">
         <v>0</v>
       </c>
@@ -32769,7 +32655,6 @@
           <t>PECAM1,VWF,KDR,CDH5,ENG</t>
         </is>
       </c>
-      <c r="N26" t="inlineStr"/>
       <c r="O26" t="n">
         <v>0</v>
       </c>
@@ -32866,7 +32751,6 @@
           <t>S100A8,S100A9,FCGR3B,CXCR2,CSF3R</t>
         </is>
       </c>
-      <c r="N27" t="inlineStr"/>
       <c r="O27" t="n">
         <v>0</v>
       </c>
@@ -32963,7 +32847,6 @@
           <t>IFNG,CXCL9,CXCL10,STAT1,IRF1,IDO1,CD274</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr"/>
       <c r="O28" t="n">
         <v>0</v>
       </c>
@@ -33060,7 +32943,6 @@
           <t>PIK3CA,PIK3CB,AKT1,AKT2,MTOR,RPS6KB1,EIF4EBP1</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
       <c r="O29" t="n">
         <v>0</v>
       </c>
@@ -33258,7 +33140,6 @@
           <t>VIM,SNAI1,SNAI2,ZEB1,ZEB2,CDH2,FN1,ITGA5,MMP2</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr"/>
       <c r="O31" t="n">
         <v>0</v>
       </c>
@@ -33456,7 +33337,6 @@
           <t>HIF1A,VEGFA,CA9,SLC2A1,LDHA,PDK1</t>
         </is>
       </c>
-      <c r="N33" t="inlineStr"/>
       <c r="O33" t="n">
         <v>0</v>
       </c>
@@ -33553,7 +33433,6 @@
           <t>MKI67,PCNA,TOP2A,CCNB1,MCM2,MCM6</t>
         </is>
       </c>
-      <c r="N34" t="inlineStr"/>
       <c r="O34" t="n">
         <v>0</v>
       </c>
@@ -33650,7 +33529,6 @@
           <t>BAX,CASP3,CASP8,FAS,BCL2L11,PMAIP1</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
       <c r="O35" t="n">
         <v>0</v>
       </c>
@@ -33747,7 +33625,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr"/>
       <c r="O36" t="n">
         <v>0</v>
       </c>
@@ -33844,7 +33721,6 @@
           <t>CD274,PDCD1,CTLA4,LAG3,TIGIT,HAVCR2</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr"/>
       <c r="O37" t="n">
         <v>0</v>
       </c>
@@ -33941,7 +33817,6 @@
           <t>CD8A,CD8B,GZMB,PRF1,NKG7,GNLY</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr"/>
       <c r="O38" t="n">
         <v>0</v>
       </c>
@@ -34038,7 +33913,6 @@
           <t>FOXP3,IL2RA,CTLA4,IKZF2,CCR8</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr"/>
       <c r="O39" t="n">
         <v>0</v>
       </c>
@@ -34135,7 +34009,6 @@
           <t>PDCD1,CD274,CTLA4,LAG3,HAVCR2,TIGIT</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr"/>
       <c r="O40" t="n">
         <v>0</v>
       </c>
@@ -34232,7 +34105,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N41" t="inlineStr"/>
       <c r="O41" t="n">
         <v>0</v>
       </c>
@@ -34329,7 +34201,6 @@
           <t>CD68,CD163,MRC1,CSF1R,MSR1</t>
         </is>
       </c>
-      <c r="N42" t="inlineStr"/>
       <c r="O42" t="n">
         <v>0</v>
       </c>
@@ -34426,7 +34297,6 @@
           <t>FAP,ACTA2,COL1A1,COL1A2,PDGFRB,POSTN</t>
         </is>
       </c>
-      <c r="N43" t="inlineStr"/>
       <c r="O43" t="n">
         <v>0</v>
       </c>
@@ -34523,7 +34393,6 @@
           <t>PECAM1,VWF,KDR,CDH5,ENG</t>
         </is>
       </c>
-      <c r="N44" t="inlineStr"/>
       <c r="O44" t="n">
         <v>0</v>
       </c>
@@ -34620,7 +34489,6 @@
           <t>S100A8,S100A9,FCGR3B,CXCR2,CSF3R</t>
         </is>
       </c>
-      <c r="N45" t="inlineStr"/>
       <c r="O45" t="n">
         <v>0</v>
       </c>
@@ -34717,7 +34585,6 @@
           <t>IFNG,CXCL9,CXCL10,STAT1,IRF1,IDO1,CD274</t>
         </is>
       </c>
-      <c r="N46" t="inlineStr"/>
       <c r="O46" t="n">
         <v>0</v>
       </c>
@@ -35016,7 +34883,6 @@
           <t>VIM,SNAI1,SNAI2,ZEB1,ZEB2,CDH2,FN1,ITGA5,MMP2</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr"/>
       <c r="O49" t="n">
         <v>0</v>
       </c>
@@ -35113,7 +34979,6 @@
           <t>COL1A1,COL1A2,COL3A1,FN1,POSTN,LOX,MMP2,MMP9</t>
         </is>
       </c>
-      <c r="N50" t="inlineStr"/>
       <c r="O50" t="n">
         <v>0</v>
       </c>
@@ -35210,7 +35075,6 @@
           <t>HIF1A,VEGFA,CA9,SLC2A1,LDHA,PDK1</t>
         </is>
       </c>
-      <c r="N51" t="inlineStr"/>
       <c r="O51" t="n">
         <v>0</v>
       </c>
@@ -35307,7 +35171,6 @@
           <t>MKI67,PCNA,TOP2A,CCNB1,MCM2,MCM6</t>
         </is>
       </c>
-      <c r="N52" t="inlineStr"/>
       <c r="O52" t="n">
         <v>0</v>
       </c>
@@ -35404,7 +35267,6 @@
           <t>BAX,CASP3,CASP8,FAS,BCL2L11,PMAIP1</t>
         </is>
       </c>
-      <c r="N53" t="inlineStr"/>
       <c r="O53" t="n">
         <v>0</v>
       </c>
@@ -35501,7 +35363,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N54" t="inlineStr"/>
       <c r="O54" t="n">
         <v>0</v>
       </c>
@@ -35598,7 +35459,6 @@
           <t>CD274,PDCD1,CTLA4,LAG3,TIGIT,HAVCR2</t>
         </is>
       </c>
-      <c r="N55" t="inlineStr"/>
       <c r="O55" t="n">
         <v>0</v>
       </c>
@@ -35695,7 +35555,6 @@
           <t>CD8A,CD8B,GZMB,PRF1,NKG7,GNLY</t>
         </is>
       </c>
-      <c r="N56" t="inlineStr"/>
       <c r="O56" t="n">
         <v>0</v>
       </c>
@@ -35792,7 +35651,6 @@
           <t>FOXP3,IL2RA,CTLA4,IKZF2,CCR8</t>
         </is>
       </c>
-      <c r="N57" t="inlineStr"/>
       <c r="O57" t="n">
         <v>0</v>
       </c>
@@ -35889,7 +35747,6 @@
           <t>PDCD1,CD274,CTLA4,LAG3,HAVCR2,TIGIT</t>
         </is>
       </c>
-      <c r="N58" t="inlineStr"/>
       <c r="O58" t="n">
         <v>0</v>
       </c>
@@ -35986,7 +35843,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N59" t="inlineStr"/>
       <c r="O59" t="n">
         <v>0</v>
       </c>
@@ -36083,7 +35939,6 @@
           <t>CD68,CD163,MRC1,CSF1R,MSR1</t>
         </is>
       </c>
-      <c r="N60" t="inlineStr"/>
       <c r="O60" t="n">
         <v>0</v>
       </c>
@@ -36281,7 +36136,6 @@
           <t>PECAM1,VWF,KDR,CDH5,ENG</t>
         </is>
       </c>
-      <c r="N62" t="inlineStr"/>
       <c r="O62" t="n">
         <v>0</v>
       </c>
@@ -36378,7 +36232,6 @@
           <t>S100A8,S100A9,FCGR3B,CXCR2,CSF3R</t>
         </is>
       </c>
-      <c r="N63" t="inlineStr"/>
       <c r="O63" t="n">
         <v>0</v>
       </c>
@@ -36475,7 +36328,6 @@
           <t>IFNG,CXCL9,CXCL10,STAT1,IRF1,IDO1,CD274</t>
         </is>
       </c>
-      <c r="N64" t="inlineStr"/>
       <c r="O64" t="n">
         <v>0</v>
       </c>
@@ -36572,7 +36424,6 @@
           <t>PIK3CA,PIK3CB,AKT1,AKT2,MTOR,RPS6KB1,EIF4EBP1</t>
         </is>
       </c>
-      <c r="N65" t="inlineStr"/>
       <c r="O65" t="n">
         <v>0</v>
       </c>
@@ -36770,7 +36621,6 @@
           <t>VIM,SNAI1,SNAI2,ZEB1,ZEB2,CDH2,FN1,ITGA5,MMP2</t>
         </is>
       </c>
-      <c r="N67" t="inlineStr"/>
       <c r="O67" t="n">
         <v>0</v>
       </c>
@@ -36968,7 +36818,6 @@
           <t>HIF1A,VEGFA,CA9,SLC2A1,LDHA,PDK1</t>
         </is>
       </c>
-      <c r="N69" t="inlineStr"/>
       <c r="O69" t="n">
         <v>0</v>
       </c>
@@ -37065,7 +36914,6 @@
           <t>MKI67,PCNA,TOP2A,CCNB1,MCM2,MCM6</t>
         </is>
       </c>
-      <c r="N70" t="inlineStr"/>
       <c r="O70" t="n">
         <v>0</v>
       </c>
@@ -37162,7 +37010,6 @@
           <t>BAX,CASP3,CASP8,FAS,BCL2L11,PMAIP1</t>
         </is>
       </c>
-      <c r="N71" t="inlineStr"/>
       <c r="O71" t="n">
         <v>0</v>
       </c>
@@ -37259,7 +37106,6 @@
           <t>MS4A1,CD79A,CD79B,CD19,CXCL13,BANK1,PAX5</t>
         </is>
       </c>
-      <c r="N72" t="inlineStr"/>
       <c r="O72" t="n">
         <v>0</v>
       </c>
@@ -37356,7 +37202,6 @@
           <t>CD274,PDCD1,CTLA4,LAG3,TIGIT,HAVCR2</t>
         </is>
       </c>
-      <c r="N73" t="inlineStr"/>
       <c r="O73" t="n">
         <v>0</v>
       </c>
@@ -37503,8 +37348,6 @@
           <t>98 accepted probe rows</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>0 unique accepted sequences</t>
@@ -43338,7 +43181,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\results\tables\deep_axis_tcga_immune_associations.tsv</t>
+          <t>project-root:\spatial_escc_workflow\results\tables\deep_axis_tcga_immune_associations.tsv</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -43398,7 +43241,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\geo\GSE47404\GSE47404_series_matrix.txt.gz</t>
+          <t>project-root:\spatial_escc_workflow\data\geo\GSE47404\GSE47404_series_matrix.txt.gz</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -43458,7 +43301,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\geo\GSE53625\GSE53625_series_matrix.txt.gz</t>
+          <t>project-root:\spatial_escc_workflow\data\geo\GSE53625\GSE53625_series_matrix.txt.gz</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -43518,7 +43361,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\geo\GSE53625\GSM1296956_first_raw_member.txt.gz</t>
+          <t>project-root:\spatial_escc_workflow\data\geo\GSE53625\GSM1296956_first_raw_member.txt.gz</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -43578,7 +43421,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\results\tables\gse53625_ensembl_sequence_index.tsv</t>
+          <t>project-root:\spatial_escc_workflow\results\tables\gse53625_ensembl_sequence_index.tsv</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -43638,7 +43481,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\open_source_tables\HRA003627_NatCommun2023_source_data.xlsx</t>
+          <t>project-root:\spatial_escc_workflow\data\open_source_tables\HRA003627_NatCommun2023_source_data.xlsx</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -43698,7 +43541,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\open_source_tables\HRA008846_TableS3_DEG.xlsx</t>
+          <t>project-root:\spatial_escc_workflow\data\open_source_tables\HRA008846_TableS3_DEG.xlsx</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -43758,7 +43601,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\open_source_tables\HRA008846_TableS4_cell_abundance.xlsx</t>
+          <t>project-root:\spatial_escc_workflow\data\open_source_tables\HRA008846_TableS4_cell_abundance.xlsx</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -43818,7 +43661,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\open_source_tables\HRA008846_TableS6_ligand_receptor.xlsx</t>
+          <t>project-root:\spatial_escc_workflow\data\open_source_tables\HRA008846_TableS6_ligand_receptor.xlsx</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -43878,7 +43721,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>D:\codex旗下文件\可变剪接基因筛选\spatial_escc_workflow\data\gdsc\GDSC2_fitted_dose_response_27Oct23.xlsx</t>
+          <t>project-root:\spatial_escc_workflow\data\gdsc\GDSC2_fitted_dose_response_27Oct23.xlsx</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">

</xml_diff>